<commit_message>
fix: correct Excel row and column mappings for rental worksheet
Shift property columns from F–O to E–N and field rows down by
one (e.g. property_address from row 6 to 5, rents_received from
12 to 11, etc.) to match the actual template layout. Also adds a
detailed worksheet layout docstring to write_excel.py, updates
reference.md field-to-row mapping accordingly, and refreshes the
Excel template binary.
</commit_message>
<xml_diff>
--- a/Rental_Income_Worksheet_Template.xlsx
+++ b/Rental_Income_Worksheet_Template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AAA-110\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\AAA-110\Coding\schedule-e-rental-income-automator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7FDFAAC7-00D4-4F7F-9350-6DEF79CC17A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D195AA41-AB00-4275-B977-505356B801CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="894" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
     <definedName name="YRP2B">Data_Income!$B$16</definedName>
     <definedName name="YRP2E">Data_Income!$B$17</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -5689,13 +5689,13 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
-      <xdr:col>3</xdr:col>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>481853</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>22413</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
+      <xdr:col>2</xdr:col>
       <xdr:colOff>2667000</xdr:colOff>
       <xdr:row>4</xdr:row>
       <xdr:rowOff>1098767</xdr:rowOff>
@@ -5727,8 +5727,8 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1919262" y="559277"/>
-          <a:ext cx="2185147" cy="1872990"/>
+          <a:off x="1747317" y="566699"/>
+          <a:ext cx="2185147" cy="1892782"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -6027,21 +6027,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="B1:O41"/>
+  <dimension ref="A1:N41"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="21"/>
   <cols>
-    <col min="1" max="1" width="2.28515625" customWidth="1"/>
-    <col min="2" max="2" width="7.42578125" customWidth="1"/>
-    <col min="3" max="3" width="11.7109375" customWidth="1"/>
-    <col min="4" max="4" width="71.28515625" customWidth="1"/>
-    <col min="5" max="5" width="13.85546875" style="183" customWidth="1"/>
-    <col min="6" max="15" width="22" customWidth="1"/>
+    <col min="1" max="1" width="7.42578125" customWidth="1"/>
+    <col min="2" max="2" width="11.7109375" customWidth="1"/>
+    <col min="3" max="3" width="71.28515625" customWidth="1"/>
+    <col min="4" max="4" width="13.85546875" style="183" customWidth="1"/>
+    <col min="5" max="14" width="22" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:15" ht="19.5" customHeight="1">
-      <c r="B1" s="252" t="s">
+    <row r="1" spans="1:14" ht="19.5" customHeight="1">
+      <c r="A1" s="252" t="s">
         <v>6</v>
       </c>
+      <c r="B1" s="253"/>
       <c r="C1" s="253"/>
       <c r="D1" s="253"/>
       <c r="E1" s="253"/>
@@ -6053,13 +6053,13 @@
       <c r="K1" s="253"/>
       <c r="L1" s="253"/>
       <c r="M1" s="253"/>
-      <c r="N1" s="253"/>
-      <c r="O1" s="254"/>
-    </row>
-    <row r="2" spans="2:15" ht="23.25">
-      <c r="B2" s="255" t="s">
+      <c r="N1" s="254"/>
+    </row>
+    <row r="2" spans="1:14" ht="24" thickBot="1">
+      <c r="A2" s="255" t="s">
         <v>7</v>
       </c>
+      <c r="B2" s="256"/>
       <c r="C2" s="256"/>
       <c r="D2" s="256"/>
       <c r="E2" s="256"/>
@@ -6071,15 +6071,17 @@
       <c r="K2" s="256"/>
       <c r="L2" s="256"/>
       <c r="M2" s="256"/>
-      <c r="N2" s="256"/>
-      <c r="O2" s="257"/>
-    </row>
-    <row r="3" spans="2:15">
-      <c r="B3" s="258"/>
-      <c r="C3" s="259"/>
-      <c r="D3" s="260"/>
-      <c r="E3" s="315" t="s">
+      <c r="N2" s="257"/>
+    </row>
+    <row r="3" spans="1:14">
+      <c r="A3" s="258"/>
+      <c r="B3" s="259"/>
+      <c r="C3" s="260"/>
+      <c r="D3" s="315" t="s">
         <v>8</v>
+      </c>
+      <c r="E3" s="267" t="s">
+        <v>9</v>
       </c>
       <c r="F3" s="267" t="s">
         <v>9</v>
@@ -6108,15 +6110,13 @@
       <c r="N3" s="267" t="s">
         <v>9</v>
       </c>
-      <c r="O3" s="267" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="4" spans="2:15" ht="42.75" customHeight="1">
-      <c r="B4" s="185"/>
-      <c r="C4" s="186"/>
-      <c r="D4" s="187"/>
-      <c r="E4" s="316"/>
+    </row>
+    <row r="4" spans="1:14" ht="42.75" customHeight="1" thickBot="1">
+      <c r="A4" s="185"/>
+      <c r="B4" s="186"/>
+      <c r="C4" s="187"/>
+      <c r="D4" s="316"/>
+      <c r="E4" s="268"/>
       <c r="F4" s="268"/>
       <c r="G4" s="268"/>
       <c r="H4" s="268"/>
@@ -6126,13 +6126,13 @@
       <c r="L4" s="268"/>
       <c r="M4" s="268"/>
       <c r="N4" s="268"/>
-      <c r="O4" s="268"/>
-    </row>
-    <row r="5" spans="2:15" ht="90" customHeight="1">
-      <c r="B5" s="188"/>
-      <c r="C5" s="189"/>
-      <c r="D5" s="190"/>
-      <c r="E5" s="317"/>
+    </row>
+    <row r="5" spans="1:14" ht="90" customHeight="1" thickBot="1">
+      <c r="A5" s="188"/>
+      <c r="B5" s="189"/>
+      <c r="C5" s="190"/>
+      <c r="D5" s="317"/>
+      <c r="E5" s="184"/>
       <c r="F5" s="184"/>
       <c r="G5" s="184"/>
       <c r="H5" s="184"/>
@@ -6142,12 +6142,12 @@
       <c r="L5" s="184"/>
       <c r="M5" s="184"/>
       <c r="N5" s="184"/>
-      <c r="O5" s="184"/>
-    </row>
-    <row r="6" spans="2:15">
-      <c r="B6" s="261" t="s">
+    </row>
+    <row r="6" spans="1:14">
+      <c r="A6" s="261" t="s">
         <v>10</v>
       </c>
+      <c r="B6" s="262"/>
       <c r="C6" s="262"/>
       <c r="D6" s="262"/>
       <c r="E6" s="262"/>
@@ -6159,13 +6159,13 @@
       <c r="K6" s="262"/>
       <c r="L6" s="262"/>
       <c r="M6" s="262"/>
-      <c r="N6" s="262"/>
-      <c r="O6" s="263"/>
-    </row>
-    <row r="7" spans="2:15" ht="24" customHeight="1">
-      <c r="B7" s="264" t="s">
+      <c r="N6" s="263"/>
+    </row>
+    <row r="7" spans="1:14" ht="24" customHeight="1" thickBot="1">
+      <c r="A7" s="264" t="s">
         <v>11</v>
       </c>
+      <c r="B7" s="265"/>
       <c r="C7" s="265"/>
       <c r="D7" s="265"/>
       <c r="E7" s="265"/>
@@ -6177,33 +6177,33 @@
       <c r="K7" s="265"/>
       <c r="L7" s="265"/>
       <c r="M7" s="265"/>
-      <c r="N7" s="265"/>
-      <c r="O7" s="266"/>
-    </row>
-    <row r="8" spans="2:15" ht="42.75" customHeight="1">
-      <c r="B8" s="332" t="s">
+      <c r="N7" s="266"/>
+    </row>
+    <row r="8" spans="1:14" ht="42.75" customHeight="1" thickBot="1">
+      <c r="A8" s="332" t="s">
         <v>12</v>
       </c>
-      <c r="C8" s="333"/>
-      <c r="D8" s="334"/>
-      <c r="E8" s="191" t="s">
+      <c r="B8" s="333"/>
+      <c r="C8" s="334"/>
+      <c r="D8" s="191" t="s">
         <v>13</v>
       </c>
-      <c r="F8" s="192"/>
-      <c r="G8" s="193"/>
+      <c r="E8" s="192"/>
+      <c r="F8" s="193"/>
+      <c r="G8" s="194"/>
       <c r="H8" s="194"/>
       <c r="I8" s="194"/>
       <c r="J8" s="194"/>
       <c r="K8" s="194"/>
       <c r="L8" s="194"/>
       <c r="M8" s="194"/>
-      <c r="N8" s="194"/>
-      <c r="O8" s="193"/>
-    </row>
-    <row r="9" spans="2:15" ht="30.75" customHeight="1">
-      <c r="B9" s="345" t="s">
+      <c r="N8" s="193"/>
+    </row>
+    <row r="9" spans="1:14" ht="30.75" customHeight="1" thickBot="1">
+      <c r="A9" s="345" t="s">
         <v>14</v>
       </c>
+      <c r="B9" s="346"/>
       <c r="C9" s="346"/>
       <c r="D9" s="346"/>
       <c r="E9" s="346"/>
@@ -6215,13 +6215,13 @@
       <c r="K9" s="346"/>
       <c r="L9" s="346"/>
       <c r="M9" s="346"/>
-      <c r="N9" s="346"/>
-      <c r="O9" s="347"/>
-    </row>
-    <row r="10" spans="2:15" ht="24.75" customHeight="1">
-      <c r="B10" s="348" t="s">
+      <c r="N9" s="347"/>
+    </row>
+    <row r="10" spans="1:14" ht="24.75" customHeight="1" thickBot="1">
+      <c r="A10" s="348" t="s">
         <v>15</v>
       </c>
+      <c r="B10" s="349"/>
       <c r="C10" s="349"/>
       <c r="D10" s="349"/>
       <c r="E10" s="349"/>
@@ -6233,221 +6233,224 @@
       <c r="K10" s="349"/>
       <c r="L10" s="349"/>
       <c r="M10" s="349"/>
-      <c r="N10" s="349"/>
-      <c r="O10" s="350"/>
-    </row>
-    <row r="11" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B11" s="195" t="s">
+      <c r="N10" s="350"/>
+    </row>
+    <row r="11" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A11" s="195" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="272" t="s">
+      <c r="B11" s="272" t="s">
         <v>17</v>
       </c>
-      <c r="D11" s="273"/>
-      <c r="E11" s="196" t="s">
+      <c r="C11" s="273"/>
+      <c r="D11" s="196" t="s">
         <v>8</v>
       </c>
-      <c r="F11" s="197"/>
+      <c r="E11" s="197"/>
+      <c r="F11" s="198"/>
       <c r="G11" s="198"/>
-      <c r="H11" s="198"/>
+      <c r="H11" s="233"/>
       <c r="I11" s="233"/>
       <c r="J11" s="233"/>
       <c r="K11" s="233"/>
       <c r="L11" s="233"/>
       <c r="M11" s="233"/>
       <c r="N11" s="233"/>
-      <c r="O11" s="233"/>
-    </row>
-    <row r="12" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B12" s="199" t="s">
+    </row>
+    <row r="12" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A12" s="199" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="272" t="s">
+      <c r="B12" s="272" t="s">
         <v>19</v>
       </c>
-      <c r="D12" s="273"/>
-      <c r="E12" s="200" t="s">
+      <c r="C12" s="273"/>
+      <c r="D12" s="200" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="201"/>
+      <c r="E12" s="201"/>
+      <c r="F12" s="198"/>
       <c r="G12" s="198"/>
-      <c r="H12" s="198"/>
+      <c r="H12" s="233"/>
       <c r="I12" s="233"/>
       <c r="J12" s="233"/>
       <c r="K12" s="233"/>
       <c r="L12" s="233"/>
       <c r="M12" s="233"/>
       <c r="N12" s="233"/>
-      <c r="O12" s="233"/>
-    </row>
-    <row r="13" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B13" s="199" t="s">
+    </row>
+    <row r="13" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A13" s="199" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="272" t="s">
+      <c r="B13" s="272" t="s">
         <v>22</v>
       </c>
-      <c r="D13" s="273"/>
-      <c r="E13" s="200" t="s">
+      <c r="C13" s="273"/>
+      <c r="D13" s="200" t="s">
         <v>23</v>
       </c>
-      <c r="F13" s="201"/>
+      <c r="E13" s="201"/>
+      <c r="F13" s="198"/>
       <c r="G13" s="198"/>
-      <c r="H13" s="198"/>
+      <c r="H13" s="233"/>
       <c r="I13" s="233"/>
       <c r="J13" s="233"/>
       <c r="K13" s="233"/>
       <c r="L13" s="233"/>
       <c r="M13" s="233"/>
       <c r="N13" s="233"/>
-      <c r="O13" s="233"/>
-    </row>
-    <row r="14" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B14" s="199" t="s">
+    </row>
+    <row r="14" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A14" s="199" t="s">
         <v>24</v>
       </c>
-      <c r="C14" s="272" t="s">
+      <c r="B14" s="272" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="273"/>
-      <c r="E14" s="200" t="s">
+      <c r="C14" s="273"/>
+      <c r="D14" s="200" t="s">
         <v>23</v>
       </c>
-      <c r="F14" s="201"/>
+      <c r="E14" s="201"/>
+      <c r="F14" s="198"/>
       <c r="G14" s="198"/>
-      <c r="H14" s="198"/>
+      <c r="H14" s="233"/>
       <c r="I14" s="233"/>
       <c r="J14" s="233"/>
       <c r="K14" s="233"/>
       <c r="L14" s="233"/>
       <c r="M14" s="233"/>
       <c r="N14" s="233"/>
-      <c r="O14" s="233"/>
-    </row>
-    <row r="15" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B15" s="199" t="s">
+    </row>
+    <row r="15" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A15" s="199" t="s">
         <v>26</v>
       </c>
-      <c r="C15" s="272" t="s">
+      <c r="B15" s="272" t="s">
         <v>27</v>
       </c>
-      <c r="D15" s="273"/>
-      <c r="E15" s="200" t="s">
+      <c r="C15" s="273"/>
+      <c r="D15" s="200" t="s">
         <v>23</v>
       </c>
-      <c r="F15" s="201"/>
+      <c r="E15" s="201"/>
+      <c r="F15" s="198"/>
       <c r="G15" s="198"/>
-      <c r="H15" s="198"/>
+      <c r="H15" s="233"/>
       <c r="I15" s="233"/>
       <c r="J15" s="233"/>
       <c r="K15" s="233"/>
       <c r="L15" s="233"/>
       <c r="M15" s="233"/>
       <c r="N15" s="233"/>
-      <c r="O15" s="233"/>
-    </row>
-    <row r="16" spans="2:15" ht="18.75" customHeight="1">
-      <c r="B16" s="311" t="s">
+    </row>
+    <row r="16" spans="1:14" ht="18.75" customHeight="1">
+      <c r="A16" s="311" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="202" t="s">
+      <c r="B16" s="202" t="s">
         <v>29</v>
       </c>
-      <c r="D16" s="203"/>
-      <c r="E16" s="318" t="s">
+      <c r="C16" s="203"/>
+      <c r="D16" s="318" t="s">
         <v>23</v>
       </c>
-      <c r="F16" s="335"/>
+      <c r="E16" s="335"/>
+      <c r="F16" s="341"/>
       <c r="G16" s="341"/>
       <c r="H16" s="341"/>
-      <c r="I16" s="341"/>
+      <c r="I16" s="352"/>
       <c r="J16" s="352"/>
-      <c r="K16" s="352"/>
+      <c r="K16" s="341"/>
       <c r="L16" s="341"/>
       <c r="M16" s="341"/>
-      <c r="N16" s="341"/>
-      <c r="O16" s="354"/>
-    </row>
-    <row r="17" spans="2:15" ht="43.5" customHeight="1">
-      <c r="B17" s="312"/>
-      <c r="C17" s="330" t="s">
+      <c r="N16" s="354"/>
+    </row>
+    <row r="17" spans="1:14" ht="43.5" customHeight="1" thickBot="1">
+      <c r="A17" s="312"/>
+      <c r="B17" s="330" t="s">
         <v>30</v>
       </c>
-      <c r="D17" s="331"/>
-      <c r="E17" s="319"/>
-      <c r="F17" s="336"/>
+      <c r="C17" s="331"/>
+      <c r="D17" s="319"/>
+      <c r="E17" s="336"/>
+      <c r="F17" s="342"/>
       <c r="G17" s="342"/>
       <c r="H17" s="342"/>
-      <c r="I17" s="342"/>
+      <c r="I17" s="353"/>
       <c r="J17" s="353"/>
-      <c r="K17" s="353"/>
+      <c r="K17" s="342"/>
       <c r="L17" s="342"/>
       <c r="M17" s="342"/>
-      <c r="N17" s="342"/>
-      <c r="O17" s="355"/>
-    </row>
-    <row r="18" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B18" s="199" t="s">
+      <c r="N17" s="355"/>
+    </row>
+    <row r="18" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A18" s="199" t="s">
         <v>31</v>
       </c>
-      <c r="C18" s="272" t="s">
+      <c r="B18" s="272" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="273"/>
-      <c r="E18" s="200" t="s">
+      <c r="C18" s="273"/>
+      <c r="D18" s="200" t="s">
         <v>23</v>
       </c>
-      <c r="F18" s="201"/>
+      <c r="E18" s="201"/>
+      <c r="F18" s="198"/>
       <c r="G18" s="198"/>
-      <c r="H18" s="198"/>
+      <c r="H18" s="233"/>
       <c r="I18" s="233"/>
       <c r="J18" s="233"/>
       <c r="K18" s="233"/>
       <c r="L18" s="233"/>
       <c r="M18" s="233"/>
       <c r="N18" s="233"/>
-      <c r="O18" s="233"/>
-    </row>
-    <row r="19" spans="2:15" ht="66" customHeight="1">
-      <c r="B19" s="199" t="s">
+    </row>
+    <row r="19" spans="1:14" ht="66" customHeight="1" thickBot="1">
+      <c r="A19" s="199" t="s">
         <v>33</v>
       </c>
-      <c r="C19" s="272" t="s">
+      <c r="B19" s="272" t="s">
         <v>34</v>
       </c>
-      <c r="D19" s="273"/>
-      <c r="E19" s="200" t="s">
+      <c r="C19" s="273"/>
+      <c r="D19" s="200" t="s">
         <v>23</v>
       </c>
-      <c r="F19" s="201"/>
+      <c r="E19" s="201"/>
+      <c r="F19" s="198"/>
       <c r="G19" s="198"/>
-      <c r="H19" s="198"/>
+      <c r="H19" s="233"/>
       <c r="I19" s="233"/>
       <c r="J19" s="233"/>
       <c r="K19" s="233"/>
       <c r="L19" s="233"/>
       <c r="M19" s="233"/>
       <c r="N19" s="233"/>
-      <c r="O19" s="233"/>
-    </row>
-    <row r="20" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B20" s="204"/>
-      <c r="C20" s="272" t="s">
+    </row>
+    <row r="20" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A20" s="204"/>
+      <c r="B20" s="272" t="s">
         <v>35</v>
       </c>
-      <c r="D20" s="273"/>
-      <c r="E20" s="200" t="s">
+      <c r="C20" s="273"/>
+      <c r="D20" s="200" t="s">
         <v>5</v>
       </c>
-      <c r="F20" s="205">
-        <f>SUM(F11,F13:F19)-F12</f>
+      <c r="E20" s="205">
+        <f>SUM(E11,E13:E19)-E12</f>
         <v>0</v>
       </c>
+      <c r="F20" s="206">
+        <f t="shared" ref="F20:N20" si="0">SUM(F11,F13:F19)-F12</f>
+        <v>0</v>
+      </c>
       <c r="G20" s="206">
-        <f t="shared" ref="G20:O20" si="0">SUM(G11,G13:G19)-G12</f>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H20" s="206">
+      <c r="H20" s="207">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -6475,23 +6478,23 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="O20" s="207">
-        <f t="shared" si="0"/>
+    </row>
+    <row r="21" spans="1:14" ht="37.5" customHeight="1" thickBot="1">
+      <c r="A21" s="199" t="s">
+        <v>36</v>
+      </c>
+      <c r="B21" s="274" t="s">
+        <v>37</v>
+      </c>
+      <c r="C21" s="275"/>
+      <c r="D21" s="200" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" s="205">
+        <f>E8</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="2:15" ht="37.5" customHeight="1">
-      <c r="B21" s="199" t="s">
-        <v>36</v>
-      </c>
-      <c r="C21" s="274" t="s">
-        <v>37</v>
-      </c>
-      <c r="D21" s="275"/>
-      <c r="E21" s="200" t="s">
-        <v>38</v>
-      </c>
-      <c r="F21" s="205">
+      <c r="F21" s="206">
         <f>F8</f>
         <v>0</v>
       </c>
@@ -6499,16 +6502,16 @@
         <f>G8</f>
         <v>0</v>
       </c>
-      <c r="H21" s="206">
+      <c r="H21" s="207">
         <f>H8</f>
         <v>0</v>
       </c>
       <c r="I21" s="207">
-        <f>I8</f>
+        <f t="shared" ref="I21:N21" si="1">I8</f>
         <v>0</v>
       </c>
       <c r="J21" s="207">
-        <f t="shared" ref="J21:O21" si="1">J8</f>
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
       <c r="K21" s="207">
@@ -6527,38 +6530,38 @@
         <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O21" s="207">
-        <f t="shared" si="1"/>
+    </row>
+    <row r="22" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A22" s="204"/>
+      <c r="B22" s="274" t="s">
+        <v>39</v>
+      </c>
+      <c r="C22" s="275"/>
+      <c r="D22" s="200" t="s">
+        <v>5</v>
+      </c>
+      <c r="E22" s="208">
+        <f t="shared" ref="E22:H22" si="2">IF(E21=0,0,E20/E21)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B22" s="204"/>
-      <c r="C22" s="274" t="s">
-        <v>39</v>
-      </c>
-      <c r="D22" s="275"/>
-      <c r="E22" s="200" t="s">
-        <v>5</v>
-      </c>
-      <c r="F22" s="208">
-        <f t="shared" ref="F22:I22" si="2">IF(F21=0,0,F20/F21)</f>
+      <c r="F22" s="209">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="G22" s="209">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
-      <c r="H22" s="209">
+      <c r="H22" s="234">
         <f t="shared" si="2"/>
         <v>0</v>
       </c>
       <c r="I22" s="234">
-        <f t="shared" si="2"/>
+        <f t="shared" ref="I22:N22" si="3">IF(I21=0,0,I20/I21)</f>
         <v>0</v>
       </c>
       <c r="J22" s="234">
-        <f t="shared" ref="J22:O22" si="3">IF(J21=0,0,J20/J21)</f>
+        <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K22" s="234">
@@ -6577,23 +6580,20 @@
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
-      <c r="O22" s="234">
-        <f t="shared" si="3"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="2:15" ht="20.25" customHeight="1">
-      <c r="B23" s="311" t="s">
+    </row>
+    <row r="23" spans="1:14" ht="20.25" customHeight="1">
+      <c r="A23" s="311" t="s">
         <v>40</v>
       </c>
-      <c r="C23" s="202" t="s">
+      <c r="B23" s="202" t="s">
         <v>41</v>
       </c>
-      <c r="D23" s="203"/>
-      <c r="E23" s="315" t="s">
+      <c r="C23" s="203"/>
+      <c r="D23" s="315" t="s">
         <v>20</v>
       </c>
-      <c r="F23" s="337"/>
+      <c r="E23" s="337"/>
+      <c r="F23" s="343"/>
       <c r="G23" s="343"/>
       <c r="H23" s="343"/>
       <c r="I23" s="343"/>
@@ -6601,17 +6601,17 @@
       <c r="K23" s="343"/>
       <c r="L23" s="343"/>
       <c r="M23" s="343"/>
-      <c r="N23" s="343"/>
-      <c r="O23" s="356"/>
-    </row>
-    <row r="24" spans="2:15" ht="29.25" customHeight="1">
-      <c r="B24" s="312"/>
-      <c r="C24" s="210" t="s">
+      <c r="N23" s="356"/>
+    </row>
+    <row r="24" spans="1:14" ht="29.25" customHeight="1" thickBot="1">
+      <c r="A24" s="312"/>
+      <c r="B24" s="210" t="s">
         <v>42</v>
       </c>
-      <c r="D24" s="211"/>
-      <c r="E24" s="317"/>
-      <c r="F24" s="338"/>
+      <c r="C24" s="211"/>
+      <c r="D24" s="317"/>
+      <c r="E24" s="338"/>
+      <c r="F24" s="344"/>
       <c r="G24" s="344"/>
       <c r="H24" s="344"/>
       <c r="I24" s="344"/>
@@ -6619,19 +6619,22 @@
       <c r="K24" s="344"/>
       <c r="L24" s="344"/>
       <c r="M24" s="344"/>
-      <c r="N24" s="344"/>
-      <c r="O24" s="357"/>
-    </row>
-    <row r="25" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B25" s="276" t="s">
+      <c r="N24" s="357"/>
+    </row>
+    <row r="25" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A25" s="276" t="s">
         <v>43</v>
       </c>
-      <c r="C25" s="277"/>
-      <c r="D25" s="278"/>
-      <c r="E25" s="212" t="s">
+      <c r="B25" s="277"/>
+      <c r="C25" s="278"/>
+      <c r="D25" s="212" t="s">
         <v>13</v>
       </c>
-      <c r="F25" s="213">
+      <c r="E25" s="213">
+        <f>E22-E23</f>
+        <v>0</v>
+      </c>
+      <c r="F25" s="214">
         <f>F22-F23</f>
         <v>0</v>
       </c>
@@ -6644,11 +6647,11 @@
         <v>0</v>
       </c>
       <c r="I25" s="214">
-        <f>I22-I23</f>
+        <f t="shared" ref="I25:N25" si="4">I22-I23</f>
         <v>0</v>
       </c>
       <c r="J25" s="214">
-        <f t="shared" ref="J25:O25" si="4">J22-J23</f>
+        <f t="shared" si="4"/>
         <v>0</v>
       </c>
       <c r="K25" s="214">
@@ -6667,15 +6670,12 @@
         <f t="shared" si="4"/>
         <v>0</v>
       </c>
-      <c r="O25" s="214">
-        <f t="shared" si="4"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="2:15" ht="22.5" customHeight="1">
-      <c r="B26" s="322" t="s">
+    </row>
+    <row r="26" spans="1:14" ht="22.5" customHeight="1">
+      <c r="A26" s="322" t="s">
         <v>44</v>
       </c>
+      <c r="B26" s="323"/>
       <c r="C26" s="323"/>
       <c r="D26" s="323"/>
       <c r="E26" s="323"/>
@@ -6687,13 +6687,13 @@
       <c r="K26" s="323"/>
       <c r="L26" s="323"/>
       <c r="M26" s="323"/>
-      <c r="N26" s="323"/>
-      <c r="O26" s="324"/>
-    </row>
-    <row r="27" spans="2:15" ht="27" customHeight="1">
-      <c r="B27" s="325" t="s">
+      <c r="N26" s="324"/>
+    </row>
+    <row r="27" spans="1:14" ht="27" customHeight="1" thickBot="1">
+      <c r="A27" s="325" t="s">
         <v>45</v>
       </c>
+      <c r="B27" s="326"/>
       <c r="C27" s="326"/>
       <c r="D27" s="326"/>
       <c r="E27" s="326"/>
@@ -6705,38 +6705,38 @@
       <c r="K27" s="326"/>
       <c r="L27" s="326"/>
       <c r="M27" s="326"/>
-      <c r="N27" s="326"/>
-      <c r="O27" s="327"/>
-    </row>
-    <row r="28" spans="2:15" ht="14.25" customHeight="1">
-      <c r="B28" s="313" t="s">
+      <c r="N27" s="327"/>
+    </row>
+    <row r="28" spans="1:14" ht="14.25" customHeight="1">
+      <c r="A28" s="313" t="s">
         <v>46</v>
       </c>
-      <c r="C28" s="215" t="s">
+      <c r="B28" s="215" t="s">
         <v>47</v>
       </c>
-      <c r="D28" s="216"/>
-      <c r="E28" s="320" t="s">
+      <c r="C28" s="216"/>
+      <c r="D28" s="320" t="s">
         <v>8</v>
       </c>
+      <c r="E28" s="339"/>
       <c r="F28" s="339"/>
       <c r="G28" s="339"/>
-      <c r="H28" s="339"/>
+      <c r="H28" s="351"/>
       <c r="I28" s="351"/>
       <c r="J28" s="351"/>
       <c r="K28" s="351"/>
       <c r="L28" s="351"/>
       <c r="M28" s="351"/>
-      <c r="N28" s="351"/>
-      <c r="O28" s="358"/>
-    </row>
-    <row r="29" spans="2:15" ht="21" customHeight="1">
-      <c r="B29" s="313"/>
-      <c r="C29" s="215" t="s">
+      <c r="N28" s="358"/>
+    </row>
+    <row r="29" spans="1:14" ht="21" customHeight="1">
+      <c r="A29" s="313"/>
+      <c r="B29" s="215" t="s">
         <v>48</v>
       </c>
-      <c r="D29" s="216"/>
-      <c r="E29" s="320"/>
+      <c r="C29" s="216"/>
+      <c r="D29" s="320"/>
+      <c r="E29" s="339"/>
       <c r="F29" s="339"/>
       <c r="G29" s="339"/>
       <c r="H29" s="339"/>
@@ -6745,16 +6745,16 @@
       <c r="K29" s="339"/>
       <c r="L29" s="339"/>
       <c r="M29" s="339"/>
-      <c r="N29" s="339"/>
-      <c r="O29" s="358"/>
-    </row>
-    <row r="30" spans="2:15" ht="33.75" customHeight="1">
-      <c r="B30" s="314"/>
-      <c r="C30" s="328" t="s">
+      <c r="N29" s="358"/>
+    </row>
+    <row r="30" spans="1:14" ht="33.75" customHeight="1" thickBot="1">
+      <c r="A30" s="314"/>
+      <c r="B30" s="328" t="s">
         <v>49</v>
       </c>
-      <c r="D30" s="329"/>
-      <c r="E30" s="321"/>
+      <c r="C30" s="329"/>
+      <c r="D30" s="321"/>
+      <c r="E30" s="340"/>
       <c r="F30" s="340"/>
       <c r="G30" s="340"/>
       <c r="H30" s="340"/>
@@ -6763,27 +6763,29 @@
       <c r="K30" s="340"/>
       <c r="L30" s="340"/>
       <c r="M30" s="340"/>
-      <c r="N30" s="340"/>
-      <c r="O30" s="359"/>
-    </row>
-    <row r="31" spans="2:15" ht="39" customHeight="1">
-      <c r="B31" s="217" t="s">
+      <c r="N30" s="359"/>
+    </row>
+    <row r="31" spans="1:14" ht="39" customHeight="1" thickBot="1">
+      <c r="A31" s="217" t="s">
         <v>50</v>
       </c>
-      <c r="C31" s="269" t="s">
+      <c r="B31" s="269" t="s">
         <v>51</v>
       </c>
-      <c r="D31" s="270"/>
-      <c r="E31" s="219" t="s">
+      <c r="C31" s="270"/>
+      <c r="D31" s="219" t="s">
         <v>52</v>
       </c>
-      <c r="F31" s="220" t="s">
+      <c r="E31" s="220" t="s">
         <v>53</v>
       </c>
-      <c r="G31" s="221" t="s">
+      <c r="F31" s="221" t="s">
         <v>53</v>
       </c>
-      <c r="H31" s="218" t="s">
+      <c r="G31" s="218" t="s">
+        <v>53</v>
+      </c>
+      <c r="H31" s="235" t="s">
         <v>53</v>
       </c>
       <c r="I31" s="235" t="s">
@@ -6801,31 +6803,32 @@
       <c r="M31" s="235" t="s">
         <v>53</v>
       </c>
-      <c r="N31" s="235" t="s">
+      <c r="N31" s="236" t="s">
         <v>53</v>
       </c>
-      <c r="O31" s="236" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="32" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B32" s="222"/>
-      <c r="C32" s="271" t="s">
+    </row>
+    <row r="32" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A32" s="222"/>
+      <c r="B32" s="271" t="s">
         <v>54</v>
       </c>
-      <c r="D32" s="270"/>
-      <c r="E32" s="219" t="s">
+      <c r="C32" s="270"/>
+      <c r="D32" s="219" t="s">
         <v>5</v>
       </c>
-      <c r="F32" s="224">
-        <f>F28*0.75</f>
+      <c r="E32" s="224">
+        <f>E28*0.75</f>
         <v>0</v>
       </c>
-      <c r="G32" s="225">
-        <f t="shared" ref="G32:O32" si="5">G28*0.75</f>
+      <c r="F32" s="225">
+        <f t="shared" ref="F32:N32" si="5">F28*0.75</f>
         <v>0</v>
       </c>
-      <c r="H32" s="224">
+      <c r="G32" s="224">
+        <f t="shared" si="5"/>
+        <v>0</v>
+      </c>
+      <c r="H32" s="223">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
@@ -6849,55 +6852,55 @@
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="N32" s="223">
+      <c r="N32" s="237">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="O32" s="237">
-        <f t="shared" si="5"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="2:15" ht="39.75" customHeight="1">
-      <c r="B33" s="217" t="s">
+    </row>
+    <row r="33" spans="1:14" ht="39.75" customHeight="1" thickBot="1">
+      <c r="A33" s="217" t="s">
         <v>55</v>
       </c>
-      <c r="C33" s="271" t="s">
+      <c r="B33" s="271" t="s">
         <v>56</v>
       </c>
-      <c r="D33" s="270"/>
-      <c r="E33" s="219" t="s">
+      <c r="C33" s="270"/>
+      <c r="D33" s="219" t="s">
         <v>57</v>
       </c>
-      <c r="F33" s="226"/>
-      <c r="G33" s="227"/>
-      <c r="H33" s="228"/>
+      <c r="E33" s="226"/>
+      <c r="F33" s="227"/>
+      <c r="G33" s="228"/>
+      <c r="H33" s="238"/>
       <c r="I33" s="238"/>
       <c r="J33" s="238"/>
       <c r="K33" s="238"/>
       <c r="L33" s="238"/>
       <c r="M33" s="238"/>
-      <c r="N33" s="238"/>
-      <c r="O33" s="239"/>
-    </row>
-    <row r="34" spans="2:15" ht="25.5" customHeight="1">
-      <c r="B34" s="279" t="s">
+      <c r="N33" s="239"/>
+    </row>
+    <row r="34" spans="1:14" ht="25.5" customHeight="1" thickBot="1">
+      <c r="A34" s="279" t="s">
         <v>58</v>
       </c>
-      <c r="C34" s="280"/>
-      <c r="D34" s="281"/>
-      <c r="E34" s="229" t="s">
+      <c r="B34" s="280"/>
+      <c r="C34" s="281"/>
+      <c r="D34" s="229" t="s">
         <v>13</v>
       </c>
-      <c r="F34" s="230">
-        <f t="shared" ref="F34:O34" si="6">F32-F33</f>
+      <c r="E34" s="230">
+        <f t="shared" ref="E34:N34" si="6">E32-E33</f>
         <v>0</v>
       </c>
-      <c r="G34" s="231">
+      <c r="F34" s="231">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="H34" s="230">
+      <c r="G34" s="230">
+        <f t="shared" si="6"/>
+        <v>0</v>
+      </c>
+      <c r="H34" s="240">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
@@ -6921,19 +6924,16 @@
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="N34" s="240">
+      <c r="N34" s="241">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="O34" s="241">
-        <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="2:15" ht="19.5" customHeight="1">
-      <c r="B35" s="282" t="s">
+    </row>
+    <row r="35" spans="1:14" ht="19.5" customHeight="1" thickBot="1">
+      <c r="A35" s="282" t="s">
         <v>59</v>
       </c>
+      <c r="B35" s="283"/>
       <c r="C35" s="283"/>
       <c r="D35" s="283"/>
       <c r="E35" s="283"/>
@@ -6945,20 +6945,20 @@
       <c r="K35" s="283"/>
       <c r="L35" s="283"/>
       <c r="M35" s="283"/>
-      <c r="N35" s="283"/>
-      <c r="O35" s="284"/>
-    </row>
-    <row r="36" spans="2:15" ht="69.75" customHeight="1">
-      <c r="B36" s="285" t="s">
+      <c r="N35" s="284"/>
+    </row>
+    <row r="36" spans="1:14" ht="69.75" customHeight="1" thickBot="1">
+      <c r="A36" s="285" t="s">
         <v>60</v>
       </c>
+      <c r="B36" s="286"/>
       <c r="C36" s="286"/>
-      <c r="D36" s="286"/>
-      <c r="E36" s="287"/>
-      <c r="F36" s="288" t="str">
-        <f>IF(SUM(F25:O25,F34:O34)&gt;0,SUM(F25:O25,F34:O34),"")</f>
+      <c r="D36" s="287"/>
+      <c r="E36" s="288" t="str">
+        <f>IF(SUM(E25:N25,E34:N34)&gt;0,SUM(E25:N25,E34:N34),"")</f>
         <v/>
       </c>
+      <c r="F36" s="289"/>
       <c r="G36" s="289"/>
       <c r="H36" s="289"/>
       <c r="I36" s="289"/>
@@ -6966,20 +6966,20 @@
       <c r="K36" s="289"/>
       <c r="L36" s="289"/>
       <c r="M36" s="289"/>
-      <c r="N36" s="289"/>
-      <c r="O36" s="290"/>
-    </row>
-    <row r="37" spans="2:15" ht="45.75" customHeight="1">
-      <c r="B37" s="272" t="s">
+      <c r="N36" s="290"/>
+    </row>
+    <row r="37" spans="1:14" ht="45.75" customHeight="1" thickBot="1">
+      <c r="A37" s="272" t="s">
         <v>61</v>
       </c>
-      <c r="C37" s="291"/>
-      <c r="D37" s="292"/>
-      <c r="E37" s="293"/>
-      <c r="F37" s="294" t="str">
-        <f>IF(SUM(F25:O25,F34:O34)&lt;0,SUM(F25:O25,F34:O34),"")</f>
+      <c r="B37" s="291"/>
+      <c r="C37" s="292"/>
+      <c r="D37" s="293"/>
+      <c r="E37" s="294" t="str">
+        <f>IF(SUM(E25:N25,E34:N34)&lt;0,SUM(E25:N25,E34:N34),"")</f>
         <v/>
       </c>
+      <c r="F37" s="295"/>
       <c r="G37" s="295"/>
       <c r="H37" s="295"/>
       <c r="I37" s="295"/>
@@ -6987,43 +6987,43 @@
       <c r="K37" s="295"/>
       <c r="L37" s="295"/>
       <c r="M37" s="295"/>
-      <c r="N37" s="295"/>
-      <c r="O37" s="296"/>
-    </row>
-    <row r="38" spans="2:15" ht="27.75" customHeight="1">
-      <c r="B38" s="297" t="s">
+      <c r="N37" s="296"/>
+    </row>
+    <row r="38" spans="1:14" ht="27.75" customHeight="1" thickBot="1">
+      <c r="A38" s="297" t="s">
         <v>62</v>
       </c>
-      <c r="C38" s="298"/>
-      <c r="D38" s="299" t="s">
+      <c r="B38" s="298"/>
+      <c r="C38" s="299" t="s">
         <v>63</v>
       </c>
-      <c r="E38" s="299"/>
-      <c r="F38" s="300" t="s">
+      <c r="D38" s="299"/>
+      <c r="E38" s="300" t="s">
         <v>64</v>
       </c>
+      <c r="F38" s="300"/>
       <c r="G38" s="300"/>
-      <c r="H38" s="300"/>
+      <c r="H38" s="301"/>
       <c r="I38" s="301"/>
       <c r="J38" s="301"/>
       <c r="K38" s="301"/>
       <c r="L38" s="301"/>
       <c r="M38" s="301"/>
-      <c r="N38" s="301"/>
-      <c r="O38" s="302"/>
-    </row>
-    <row r="39" spans="2:15" ht="68.25" customHeight="1">
-      <c r="B39" s="303" t="s">
+      <c r="N38" s="302"/>
+    </row>
+    <row r="39" spans="1:14" ht="68.25" customHeight="1" thickBot="1">
+      <c r="A39" s="303" t="s">
         <v>65</v>
       </c>
-      <c r="C39" s="304"/>
-      <c r="D39" s="305" t="s">
+      <c r="B39" s="304"/>
+      <c r="C39" s="305" t="s">
         <v>66</v>
       </c>
-      <c r="E39" s="304"/>
-      <c r="F39" s="306" t="s">
+      <c r="D39" s="304"/>
+      <c r="E39" s="306" t="s">
         <v>67</v>
       </c>
+      <c r="F39" s="307"/>
       <c r="G39" s="307"/>
       <c r="H39" s="307"/>
       <c r="I39" s="307"/>
@@ -7031,21 +7031,21 @@
       <c r="K39" s="307"/>
       <c r="L39" s="307"/>
       <c r="M39" s="307"/>
-      <c r="N39" s="307"/>
-      <c r="O39" s="308"/>
-    </row>
-    <row r="40" spans="2:15" ht="44.25" customHeight="1">
-      <c r="B40" s="309" t="s">
+      <c r="N39" s="308"/>
+    </row>
+    <row r="40" spans="1:14" ht="44.25" customHeight="1" thickBot="1">
+      <c r="A40" s="309" t="s">
         <v>68</v>
       </c>
-      <c r="C40" s="310"/>
-      <c r="D40" s="305" t="s">
+      <c r="B40" s="310"/>
+      <c r="C40" s="305" t="s">
         <v>69</v>
       </c>
-      <c r="E40" s="304"/>
-      <c r="F40" s="306" t="s">
+      <c r="D40" s="304"/>
+      <c r="E40" s="306" t="s">
         <v>70</v>
       </c>
+      <c r="F40" s="307"/>
       <c r="G40" s="307"/>
       <c r="H40" s="307"/>
       <c r="I40" s="307"/>
@@ -7053,133 +7053,132 @@
       <c r="K40" s="307"/>
       <c r="L40" s="307"/>
       <c r="M40" s="307"/>
-      <c r="N40" s="307"/>
-      <c r="O40" s="308"/>
-    </row>
-    <row r="41" spans="2:15">
-      <c r="B41" s="232" t="s">
+      <c r="N40" s="308"/>
+    </row>
+    <row r="41" spans="1:14">
+      <c r="A41" s="232" t="s">
         <v>71</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="88">
-    <mergeCell ref="O16:O17"/>
-    <mergeCell ref="O23:O24"/>
-    <mergeCell ref="O28:O30"/>
+    <mergeCell ref="N16:N17"/>
+    <mergeCell ref="N23:N24"/>
+    <mergeCell ref="N28:N30"/>
+    <mergeCell ref="L16:L17"/>
+    <mergeCell ref="L23:L24"/>
+    <mergeCell ref="L28:L30"/>
     <mergeCell ref="M16:M17"/>
     <mergeCell ref="M23:M24"/>
     <mergeCell ref="M28:M30"/>
-    <mergeCell ref="N16:N17"/>
-    <mergeCell ref="N23:N24"/>
-    <mergeCell ref="N28:N30"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="J23:J24"/>
+    <mergeCell ref="J28:J30"/>
     <mergeCell ref="K16:K17"/>
     <mergeCell ref="K23:K24"/>
     <mergeCell ref="K28:K30"/>
-    <mergeCell ref="L16:L17"/>
-    <mergeCell ref="L23:L24"/>
-    <mergeCell ref="L28:L30"/>
+    <mergeCell ref="H23:H24"/>
+    <mergeCell ref="H28:H30"/>
+    <mergeCell ref="I16:I17"/>
     <mergeCell ref="I23:I24"/>
     <mergeCell ref="I28:I30"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="J23:J24"/>
-    <mergeCell ref="J28:J30"/>
+    <mergeCell ref="E16:E17"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="E28:E30"/>
+    <mergeCell ref="F3:F4"/>
     <mergeCell ref="F16:F17"/>
     <mergeCell ref="F23:F24"/>
     <mergeCell ref="F28:F30"/>
-    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="A9:N9"/>
+    <mergeCell ref="A10:N10"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="B12:C12"/>
     <mergeCell ref="G16:G17"/>
     <mergeCell ref="G23:G24"/>
     <mergeCell ref="G28:G30"/>
-    <mergeCell ref="B9:O9"/>
-    <mergeCell ref="B10:O10"/>
-    <mergeCell ref="C11:D11"/>
-    <mergeCell ref="C12:D12"/>
+    <mergeCell ref="H3:H4"/>
     <mergeCell ref="H16:H17"/>
-    <mergeCell ref="H23:H24"/>
-    <mergeCell ref="H28:H30"/>
+    <mergeCell ref="A16:A17"/>
+    <mergeCell ref="A23:A24"/>
+    <mergeCell ref="A28:A30"/>
+    <mergeCell ref="D3:D5"/>
+    <mergeCell ref="D16:D17"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="D28:D30"/>
+    <mergeCell ref="A26:N26"/>
+    <mergeCell ref="A27:N27"/>
+    <mergeCell ref="B30:C30"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="B15:C15"/>
+    <mergeCell ref="B17:C17"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A39:B39"/>
+    <mergeCell ref="C39:D39"/>
+    <mergeCell ref="E39:N39"/>
+    <mergeCell ref="A40:B40"/>
+    <mergeCell ref="C40:D40"/>
+    <mergeCell ref="E40:N40"/>
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="E37:N37"/>
+    <mergeCell ref="A38:B38"/>
+    <mergeCell ref="C38:D38"/>
+    <mergeCell ref="E38:N38"/>
+    <mergeCell ref="B33:C33"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="A35:N35"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="E36:N36"/>
+    <mergeCell ref="B31:C31"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B19:C19"/>
+    <mergeCell ref="B20:C20"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="B22:C22"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A1:N1"/>
+    <mergeCell ref="A2:N2"/>
+    <mergeCell ref="A3:C3"/>
+    <mergeCell ref="A6:N6"/>
+    <mergeCell ref="A7:N7"/>
+    <mergeCell ref="E3:E4"/>
+    <mergeCell ref="G3:G4"/>
     <mergeCell ref="I3:I4"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="B23:B24"/>
-    <mergeCell ref="B28:B30"/>
-    <mergeCell ref="E3:E5"/>
-    <mergeCell ref="E16:E17"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="E28:E30"/>
-    <mergeCell ref="B26:O26"/>
-    <mergeCell ref="B27:O27"/>
-    <mergeCell ref="C30:D30"/>
-    <mergeCell ref="C13:D13"/>
-    <mergeCell ref="C14:D14"/>
-    <mergeCell ref="C15:D15"/>
-    <mergeCell ref="C17:D17"/>
-    <mergeCell ref="C18:D18"/>
-    <mergeCell ref="B8:D8"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="F39:O39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="F40:O40"/>
-    <mergeCell ref="B37:E37"/>
-    <mergeCell ref="F37:O37"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="F38:O38"/>
-    <mergeCell ref="C33:D33"/>
-    <mergeCell ref="B34:D34"/>
-    <mergeCell ref="B35:O35"/>
-    <mergeCell ref="B36:E36"/>
-    <mergeCell ref="F36:O36"/>
-    <mergeCell ref="C31:D31"/>
-    <mergeCell ref="C32:D32"/>
-    <mergeCell ref="C19:D19"/>
-    <mergeCell ref="C20:D20"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="B25:D25"/>
-    <mergeCell ref="B1:O1"/>
-    <mergeCell ref="B2:O2"/>
-    <mergeCell ref="B3:D3"/>
-    <mergeCell ref="B6:O6"/>
-    <mergeCell ref="B7:O7"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="M3:M4"/>
     <mergeCell ref="J3:J4"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="N3:N4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="M3:M4"/>
-    <mergeCell ref="O3:O4"/>
   </mergeCells>
   <phoneticPr fontId="12" type="noConversion"/>
   <dataValidations count="9">
-    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Must enter a number between 1-12" sqref="F8:O8" xr:uid="{00000000-0002-0000-0500-000000000000}">
+    <dataValidation type="whole" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Must enter a number between 1-12" sqref="E8:N8" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>1</formula1>
       <formula2>12</formula2>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="F13:O13" xr:uid="{00000000-0002-0000-0500-000001000000}">
-      <formula1>AND(F13&gt;=0,F13&lt;F12)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="E13:N13" xr:uid="{00000000-0002-0000-0500-000001000000}">
+      <formula1>AND(E13&gt;=0,E13&lt;E12)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="F14:O14" xr:uid="{00000000-0002-0000-0500-000002000000}">
-      <formula1>AND(F14&gt;=0,F14&lt;F12)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="E14:N14" xr:uid="{00000000-0002-0000-0500-000002000000}">
+      <formula1>AND(E14&gt;=0,E14&lt;E12)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="F15:O15" xr:uid="{00000000-0002-0000-0500-000003000000}">
-      <formula1>AND(F15&gt;=0,F15&lt;F12)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="E15:N15" xr:uid="{00000000-0002-0000-0500-000003000000}">
+      <formula1>AND(E15&gt;=0,E15&lt;E12)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="F18:O18" xr:uid="{00000000-0002-0000-0500-000004000000}">
-      <formula1>AND(F18&gt;=0,F18&lt;F12)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="E18:N18" xr:uid="{00000000-0002-0000-0500-000004000000}">
+      <formula1>AND(E18&gt;=0,E18&lt;E12)</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="F19:O19" xr:uid="{00000000-0002-0000-0500-000005000000}">
-      <formula1>AND(F19&gt;=0,F19&lt;F12)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="E19:N19" xr:uid="{00000000-0002-0000-0500-000005000000}">
+      <formula1>AND(E19&gt;=0,E19&lt;E12)</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Number must be positive" sqref="I23:N23 F33:O33 O23:O24 F23:H24" xr:uid="{00000000-0002-0000-0500-000006000000}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Number must be positive" sqref="H23:M23 E33:N33 N23:N24 E23:G24" xr:uid="{00000000-0002-0000-0500-000006000000}">
       <formula1>0</formula1>
     </dataValidation>
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="F16:O17" xr:uid="{00000000-0002-0000-0500-000007000000}">
-      <formula1>AND(F16&gt;=0,F16&lt;F12)</formula1>
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Positive value must be less than total expenses" sqref="E16:N17" xr:uid="{00000000-0002-0000-0500-000007000000}">
+      <formula1>AND(E16&gt;=0,E16&lt;E12)</formula1>
     </dataValidation>
-    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter a positive number" sqref="F11:O12" xr:uid="{00000000-0002-0000-0500-000008000000}">
+    <dataValidation type="whole" operator="greaterThanOrEqual" allowBlank="1" showInputMessage="1" showErrorMessage="1" error="Please enter a positive number" sqref="E11:N12" xr:uid="{00000000-0002-0000-0500-000008000000}">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>